<commit_message>
Done with all the agent
ww
</commit_message>
<xml_diff>
--- a/agent/student_attendance_TOTAL_SUMMARY.xlsx
+++ b/agent/student_attendance_TOTAL_SUMMARY.xlsx
@@ -468,10 +468,10 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D2" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
@@ -498,20 +498,20 @@
         </is>
       </c>
       <c r="C3" t="n">
+        <v>27</v>
+      </c>
+      <c r="D3" t="n">
         <v>25</v>
       </c>
-      <c r="D3" t="n">
-        <v>24</v>
-      </c>
       <c r="E3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F3" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>96.0%</t>
+          <t>92.6%</t>
         </is>
       </c>
       <c r="H3" t="n">
@@ -528,10 +528,10 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D4" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E4" t="n">
         <v>0</v>
@@ -558,16 +558,16 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D5" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E5" t="n">
         <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -588,16 +588,16 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D6" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E6" t="n">
         <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -618,10 +618,10 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D7" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E7" t="n">
         <v>0</v>
@@ -648,16 +648,16 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D8" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E8" t="n">
         <v>0</v>
       </c>
       <c r="F8" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -678,10 +678,10 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D9" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E9" t="n">
         <v>1</v>
@@ -691,7 +691,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>96.0%</t>
+          <t>96.3%</t>
         </is>
       </c>
       <c r="H9" t="n">
@@ -708,10 +708,10 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D10" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E10" t="n">
         <v>0</v>
@@ -738,10 +738,10 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D11" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E11" t="n">
         <v>0</v>
@@ -768,10 +768,10 @@
         </is>
       </c>
       <c r="C12" t="n">
+        <v>26</v>
+      </c>
+      <c r="D12" t="n">
         <v>25</v>
-      </c>
-      <c r="D12" t="n">
-        <v>24</v>
       </c>
       <c r="E12" t="n">
         <v>1</v>
@@ -781,7 +781,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>96.0%</t>
+          <t>96.2%</t>
         </is>
       </c>
       <c r="H12" t="n">
@@ -798,20 +798,20 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D13" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E13" t="n">
         <v>0</v>
       </c>
       <c r="F13" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>100.0%</t>
         </is>
       </c>
       <c r="H13" t="n">
@@ -828,10 +828,10 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D14" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E14" t="n">
         <v>0</v>
@@ -858,10 +858,10 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D15" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E15" t="n">
         <v>1</v>
@@ -871,7 +871,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>96.0%</t>
+          <t>96.3%</t>
         </is>
       </c>
       <c r="H15" t="n">
@@ -888,16 +888,16 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D16" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E16" t="n">
         <v>0</v>
       </c>
       <c r="F16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
@@ -918,16 +918,16 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D17" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E17" t="n">
         <v>0</v>
       </c>
       <c r="F17" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
@@ -948,16 +948,16 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D18" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E18" t="n">
         <v>0</v>
       </c>
       <c r="F18" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
@@ -978,10 +978,10 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D19" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E19" t="n">
         <v>0</v>
@@ -1008,10 +1008,10 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D20" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E20" t="n">
         <v>0</v>
@@ -1038,10 +1038,10 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D21" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E21" t="n">
         <v>1</v>
@@ -1051,7 +1051,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>96.0%</t>
+          <t>96.3%</t>
         </is>
       </c>
       <c r="H21" t="n">
@@ -1068,16 +1068,16 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D22" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E22" t="n">
         <v>0</v>
       </c>
       <c r="F22" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
@@ -1098,20 +1098,20 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D23" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F23" t="n">
         <v>4</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>100.0%</t>
+          <t>96.3%</t>
         </is>
       </c>
       <c r="H23" t="n">
@@ -1128,10 +1128,10 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D24" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E24" t="n">
         <v>0</v>
@@ -1158,16 +1158,16 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D25" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E25" t="n">
         <v>0</v>
       </c>
       <c r="F25" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
@@ -1188,10 +1188,10 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D26" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E26" t="n">
         <v>0</v>
@@ -1218,10 +1218,10 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D27" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E27" t="n">
         <v>0</v>
@@ -1248,10 +1248,10 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D28" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E28" t="n">
         <v>0</v>
@@ -1308,10 +1308,10 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D30" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E30" t="n">
         <v>0</v>
@@ -1338,16 +1338,16 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D31" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E31" t="n">
         <v>0</v>
       </c>
       <c r="F31" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G31" t="inlineStr">
         <is>
@@ -1368,10 +1368,10 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D32" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E32" t="n">
         <v>0</v>
@@ -1398,10 +1398,10 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D33" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E33" t="n">
         <v>0</v>
@@ -1428,10 +1428,10 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D34" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E34" t="n">
         <v>0</v>
@@ -1458,10 +1458,10 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D35" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E35" t="n">
         <v>0</v>
@@ -1488,10 +1488,10 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D36" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E36" t="n">
         <v>1</v>
@@ -1501,7 +1501,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>96.0%</t>
+          <t>96.3%</t>
         </is>
       </c>
       <c r="H36" t="n">
@@ -1518,10 +1518,10 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D37" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E37" t="n">
         <v>0</v>
@@ -1548,10 +1548,10 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D38" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E38" t="n">
         <v>0</v>
@@ -1578,10 +1578,10 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D39" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E39" t="n">
         <v>0</v>
@@ -1608,10 +1608,10 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D40" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E40" t="n">
         <v>0</v>
@@ -1638,10 +1638,10 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D41" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E41" t="n">
         <v>0</v>
@@ -1668,16 +1668,16 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D42" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E42" t="n">
         <v>0</v>
       </c>
       <c r="F42" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G42" t="inlineStr">
         <is>
@@ -1698,16 +1698,16 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D43" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E43" t="n">
         <v>0</v>
       </c>
       <c r="F43" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G43" t="inlineStr">
         <is>
@@ -1728,16 +1728,16 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D44" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E44" t="n">
         <v>0</v>
       </c>
       <c r="F44" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G44" t="inlineStr">
         <is>
@@ -1758,16 +1758,16 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D45" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E45" t="n">
         <v>0</v>
       </c>
       <c r="F45" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G45" t="inlineStr">
         <is>
@@ -1788,10 +1788,10 @@
         </is>
       </c>
       <c r="C46" t="n">
+        <v>26</v>
+      </c>
+      <c r="D46" t="n">
         <v>25</v>
-      </c>
-      <c r="D46" t="n">
-        <v>24</v>
       </c>
       <c r="E46" t="n">
         <v>1</v>
@@ -1801,7 +1801,7 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>96.0%</t>
+          <t>96.2%</t>
         </is>
       </c>
       <c r="H46" t="n">
@@ -1818,10 +1818,10 @@
         </is>
       </c>
       <c r="C47" t="n">
+        <v>26</v>
+      </c>
+      <c r="D47" t="n">
         <v>25</v>
-      </c>
-      <c r="D47" t="n">
-        <v>24</v>
       </c>
       <c r="E47" t="n">
         <v>1</v>
@@ -1831,7 +1831,7 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>96.0%</t>
+          <t>96.2%</t>
         </is>
       </c>
       <c r="H47" t="n">
@@ -1848,10 +1848,10 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D48" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E48" t="n">
         <v>0</v>
@@ -1878,10 +1878,10 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D49" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E49" t="n">
         <v>0</v>
@@ -1908,20 +1908,20 @@
         </is>
       </c>
       <c r="C50" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D50" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E50" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F50" t="n">
         <v>7</v>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>100.0%</t>
+          <t>96.3%</t>
         </is>
       </c>
       <c r="H50" t="n">
@@ -1938,10 +1938,10 @@
         </is>
       </c>
       <c r="C51" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D51" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E51" t="n">
         <v>1</v>
@@ -1951,7 +1951,7 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>96.0%</t>
+          <t>96.3%</t>
         </is>
       </c>
       <c r="H51" t="n">
@@ -1968,10 +1968,10 @@
         </is>
       </c>
       <c r="C52" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D52" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E52" t="n">
         <v>0</v>
@@ -1998,20 +1998,20 @@
         </is>
       </c>
       <c r="C53" t="n">
+        <v>27</v>
+      </c>
+      <c r="D53" t="n">
         <v>25</v>
       </c>
-      <c r="D53" t="n">
-        <v>24</v>
-      </c>
       <c r="E53" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F53" t="n">
         <v>4</v>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>96.0%</t>
+          <t>92.6%</t>
         </is>
       </c>
       <c r="H53" t="n">
@@ -2028,10 +2028,10 @@
         </is>
       </c>
       <c r="C54" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D54" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E54" t="n">
         <v>1</v>
@@ -2041,7 +2041,7 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>96.0%</t>
+          <t>96.3%</t>
         </is>
       </c>
       <c r="H54" t="n">
@@ -2058,10 +2058,10 @@
         </is>
       </c>
       <c r="C55" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D55" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E55" t="n">
         <v>0</v>
@@ -2088,16 +2088,16 @@
         </is>
       </c>
       <c r="C56" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D56" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E56" t="n">
         <v>0</v>
       </c>
       <c r="F56" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G56" t="inlineStr">
         <is>
@@ -2118,10 +2118,10 @@
         </is>
       </c>
       <c r="C57" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D57" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E57" t="n">
         <v>0</v>
@@ -2148,16 +2148,16 @@
         </is>
       </c>
       <c r="C58" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D58" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E58" t="n">
         <v>0</v>
       </c>
       <c r="F58" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G58" t="inlineStr">
         <is>
@@ -2178,10 +2178,10 @@
         </is>
       </c>
       <c r="C59" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D59" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E59" t="n">
         <v>1</v>
@@ -2191,7 +2191,7 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>96.0%</t>
+          <t>96.3%</t>
         </is>
       </c>
       <c r="H59" t="n">
@@ -2208,16 +2208,16 @@
         </is>
       </c>
       <c r="C60" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D60" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E60" t="n">
         <v>0</v>
       </c>
       <c r="F60" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G60" t="inlineStr">
         <is>
@@ -2238,16 +2238,16 @@
         </is>
       </c>
       <c r="C61" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D61" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E61" t="n">
         <v>0</v>
       </c>
       <c r="F61" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G61" t="inlineStr">
         <is>
@@ -2268,20 +2268,20 @@
         </is>
       </c>
       <c r="C62" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D62" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E62" t="n">
         <v>0</v>
       </c>
       <c r="F62" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>100.0%</t>
         </is>
       </c>
       <c r="H62" t="n">
@@ -2298,10 +2298,10 @@
         </is>
       </c>
       <c r="C63" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D63" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E63" t="n">
         <v>0</v>
@@ -2328,10 +2328,10 @@
         </is>
       </c>
       <c r="C64" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D64" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E64" t="n">
         <v>0</v>
@@ -2388,16 +2388,16 @@
         </is>
       </c>
       <c r="C66" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D66" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E66" t="n">
         <v>0</v>
       </c>
       <c r="F66" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G66" t="inlineStr">
         <is>
@@ -2418,10 +2418,10 @@
         </is>
       </c>
       <c r="C67" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D67" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E67" t="n">
         <v>0</v>
@@ -2448,16 +2448,16 @@
         </is>
       </c>
       <c r="C68" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D68" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E68" t="n">
         <v>0</v>
       </c>
       <c r="F68" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G68" t="inlineStr">
         <is>
@@ -2478,20 +2478,20 @@
         </is>
       </c>
       <c r="C69" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D69" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E69" t="n">
         <v>1</v>
       </c>
       <c r="F69" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>96.0%</t>
+          <t>96.3%</t>
         </is>
       </c>
       <c r="H69" t="n">
@@ -2508,20 +2508,20 @@
         </is>
       </c>
       <c r="C70" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D70" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E70" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F70" t="n">
         <v>2</v>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>100.0%</t>
+          <t>96.3%</t>
         </is>
       </c>
       <c r="H70" t="n">
@@ -2538,20 +2538,20 @@
         </is>
       </c>
       <c r="C71" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D71" t="n">
         <v>25</v>
       </c>
       <c r="E71" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F71" t="n">
         <v>7</v>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>100.0%</t>
+          <t>96.2%</t>
         </is>
       </c>
       <c r="H71" t="n">
@@ -2568,10 +2568,10 @@
         </is>
       </c>
       <c r="C72" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D72" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E72" t="n">
         <v>0</v>
@@ -2598,10 +2598,10 @@
         </is>
       </c>
       <c r="C73" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D73" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E73" t="n">
         <v>0</v>
@@ -2628,16 +2628,16 @@
         </is>
       </c>
       <c r="C74" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D74" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E74" t="n">
         <v>0</v>
       </c>
       <c r="F74" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G74" t="inlineStr">
         <is>
@@ -2658,16 +2658,16 @@
         </is>
       </c>
       <c r="C75" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D75" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E75" t="n">
         <v>0</v>
       </c>
       <c r="F75" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G75" t="inlineStr">
         <is>
@@ -2688,20 +2688,20 @@
         </is>
       </c>
       <c r="C76" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D76" t="n">
         <v>25</v>
       </c>
       <c r="E76" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F76" t="n">
         <v>0</v>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>100.0%</t>
+          <t>96.2%</t>
         </is>
       </c>
       <c r="H76" t="n">
@@ -2718,16 +2718,16 @@
         </is>
       </c>
       <c r="C77" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D77" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E77" t="n">
         <v>0</v>
       </c>
       <c r="F77" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G77" t="inlineStr">
         <is>
@@ -2748,10 +2748,10 @@
         </is>
       </c>
       <c r="C78" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D78" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E78" t="n">
         <v>1</v>
@@ -2761,7 +2761,7 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>96.0%</t>
+          <t>96.3%</t>
         </is>
       </c>
       <c r="H78" t="n">
@@ -2778,16 +2778,16 @@
         </is>
       </c>
       <c r="C79" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D79" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E79" t="n">
         <v>0</v>
       </c>
       <c r="F79" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G79" t="inlineStr">
         <is>
@@ -2838,16 +2838,16 @@
         </is>
       </c>
       <c r="C81" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D81" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E81" t="n">
         <v>0</v>
       </c>
       <c r="F81" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G81" t="inlineStr">
         <is>
@@ -2868,10 +2868,10 @@
         </is>
       </c>
       <c r="C82" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D82" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E82" t="n">
         <v>0</v>
@@ -2898,10 +2898,10 @@
         </is>
       </c>
       <c r="C83" t="n">
+        <v>26</v>
+      </c>
+      <c r="D83" t="n">
         <v>25</v>
-      </c>
-      <c r="D83" t="n">
-        <v>24</v>
       </c>
       <c r="E83" t="n">
         <v>1</v>
@@ -2911,7 +2911,7 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>96.0%</t>
+          <t>96.2%</t>
         </is>
       </c>
       <c r="H83" t="n">
@@ -2928,10 +2928,10 @@
         </is>
       </c>
       <c r="C84" t="n">
+        <v>26</v>
+      </c>
+      <c r="D84" t="n">
         <v>25</v>
-      </c>
-      <c r="D84" t="n">
-        <v>24</v>
       </c>
       <c r="E84" t="n">
         <v>1</v>
@@ -2941,7 +2941,7 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>96.0%</t>
+          <t>96.2%</t>
         </is>
       </c>
       <c r="H84" t="n">
@@ -2958,10 +2958,10 @@
         </is>
       </c>
       <c r="C85" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D85" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E85" t="n">
         <v>0</v>
@@ -2988,16 +2988,16 @@
         </is>
       </c>
       <c r="C86" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D86" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E86" t="n">
         <v>0</v>
       </c>
       <c r="F86" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G86" t="inlineStr">
         <is>
@@ -3018,20 +3018,20 @@
         </is>
       </c>
       <c r="C87" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D87" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E87" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F87" t="n">
         <v>4</v>
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>100.0%</t>
+          <t>96.3%</t>
         </is>
       </c>
       <c r="H87" t="n">
@@ -3048,20 +3048,20 @@
         </is>
       </c>
       <c r="C88" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D88" t="n">
         <v>24</v>
       </c>
       <c r="E88" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F88" t="n">
         <v>5</v>
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>96.0%</t>
+          <t>92.3%</t>
         </is>
       </c>
       <c r="H88" t="n">
@@ -3078,16 +3078,16 @@
         </is>
       </c>
       <c r="C89" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D89" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E89" t="n">
         <v>0</v>
       </c>
       <c r="F89" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G89" t="inlineStr">
         <is>
@@ -3108,10 +3108,10 @@
         </is>
       </c>
       <c r="C90" t="n">
+        <v>26</v>
+      </c>
+      <c r="D90" t="n">
         <v>25</v>
-      </c>
-      <c r="D90" t="n">
-        <v>24</v>
       </c>
       <c r="E90" t="n">
         <v>1</v>
@@ -3121,7 +3121,7 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>96.0%</t>
+          <t>96.2%</t>
         </is>
       </c>
       <c r="H90" t="n">
@@ -3138,10 +3138,10 @@
         </is>
       </c>
       <c r="C91" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D91" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E91" t="n">
         <v>1</v>
@@ -3151,7 +3151,7 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>96.0%</t>
+          <t>96.3%</t>
         </is>
       </c>
       <c r="H91" t="n">
@@ -3168,10 +3168,10 @@
         </is>
       </c>
       <c r="C92" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D92" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E92" t="n">
         <v>0</v>
@@ -3198,10 +3198,10 @@
         </is>
       </c>
       <c r="C93" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D93" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E93" t="n">
         <v>0</v>
@@ -3228,10 +3228,10 @@
         </is>
       </c>
       <c r="C94" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D94" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E94" t="n">
         <v>1</v>
@@ -3241,7 +3241,7 @@
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>96.0%</t>
+          <t>96.3%</t>
         </is>
       </c>
       <c r="H94" t="n">
@@ -3258,10 +3258,10 @@
         </is>
       </c>
       <c r="C95" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D95" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E95" t="n">
         <v>0</v>
@@ -3288,16 +3288,16 @@
         </is>
       </c>
       <c r="C96" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D96" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E96" t="n">
         <v>0</v>
       </c>
       <c r="F96" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G96" t="inlineStr">
         <is>
@@ -3318,16 +3318,16 @@
         </is>
       </c>
       <c r="C97" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D97" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E97" t="n">
         <v>0</v>
       </c>
       <c r="F97" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G97" t="inlineStr">
         <is>
@@ -3348,10 +3348,10 @@
         </is>
       </c>
       <c r="C98" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D98" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E98" t="n">
         <v>0</v>
@@ -3378,10 +3378,10 @@
         </is>
       </c>
       <c r="C99" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D99" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E99" t="n">
         <v>0</v>
@@ -3408,10 +3408,10 @@
         </is>
       </c>
       <c r="C100" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D100" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E100" t="n">
         <v>0</v>
@@ -3438,20 +3438,20 @@
         </is>
       </c>
       <c r="C101" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D101" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E101" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F101" t="n">
         <v>7</v>
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>100.0%</t>
+          <t>96.3%</t>
         </is>
       </c>
       <c r="H101" t="n">

</xml_diff>